<commit_message>
stations last fix i hope
</commit_message>
<xml_diff>
--- a/_stations_info_handler/v1.xlsx
+++ b/_stations_info_handler/v1.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\carlos\01_pesquisa\meteobr\_stations_info_handler\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{34D7C4BF-09C2-4125-B4FC-CBA882F1EA5F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{153C4E3C-1137-471E-965E-18C07F15511E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3346" uniqueCount="2134">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3345" uniqueCount="2133">
   <si>
     <t>town.name</t>
   </si>
@@ -6413,9 +6413,6 @@
   </si>
   <si>
     <t>2114007</t>
-  </si>
-  <si>
-    <t>BARREIRINHAS</t>
   </si>
   <si>
     <t>TORRES</t>
@@ -18702,8 +18699,8 @@
       <c r="H412" t="s">
         <v>1588</v>
       </c>
-      <c r="I412" t="s">
-        <v>2131</v>
+      <c r="I412">
+        <v>2101707</v>
       </c>
     </row>
     <row r="413" spans="1:9" x14ac:dyDescent="0.25">
@@ -23145,13 +23142,13 @@
     </row>
     <row r="566" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A566" t="s">
-        <v>2132</v>
+        <v>2131</v>
       </c>
       <c r="B566" t="s">
         <v>47</v>
       </c>
       <c r="H566" t="s">
-        <v>2133</v>
+        <v>2132</v>
       </c>
       <c r="I566">
         <v>4321501</v>

</xml_diff>